<commit_message>
Ajour README + Ajout fichiers lib.
</commit_message>
<xml_diff>
--- a/doc/Doc_KSA/2418_DemonstrateurGraphique_Cablage.xlsx
+++ b/doc/Doc_KSA/2418_DemonstrateurGraphique_Cablage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\microchip\harmony\v2_06\apps\PROJ\PRJ_2418_demosntrateurGraphique-\doc\Doc_KSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2355E533-D3CB-496A-B65F-EB2F9E3046DD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC527DD-AB2D-46DB-9B14-C3FB30240D5B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="42">
   <si>
     <t>Pin No. Display</t>
   </si>
@@ -132,6 +132,33 @@
   </si>
   <si>
     <t>X1/X2/X3/X4</t>
+  </si>
+  <si>
+    <t>17 (RA0)</t>
+  </si>
+  <si>
+    <t>38 (RA1)</t>
+  </si>
+  <si>
+    <t>23 (RB2)</t>
+  </si>
+  <si>
+    <t>X13 Pint.1 (Output)</t>
+  </si>
+  <si>
+    <t>X13 Pin.2 (Output)</t>
+  </si>
+  <si>
+    <t>X8 Pin.3 (Input)</t>
+  </si>
+  <si>
+    <t>X17  Pin.2</t>
+  </si>
+  <si>
+    <t>&gt;</t>
+  </si>
+  <si>
+    <t>&lt;</t>
   </si>
 </sst>
 </file>
@@ -760,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D3:H21"/>
+  <dimension ref="D3:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="1"/>
@@ -768,8 +795,8 @@
     <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="4:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D4" s="11" t="s">
         <v>0</v>
       </c>
@@ -786,7 +813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D5" s="14">
         <v>1</v>
       </c>
@@ -799,9 +826,11 @@
       <c r="G5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="15"/>
-    </row>
-    <row r="6" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="H5" s="15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D6" s="16">
         <v>2</v>
       </c>
@@ -818,7 +847,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D7" s="18">
         <v>3</v>
       </c>
@@ -835,7 +864,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D8" s="20">
         <v>4</v>
       </c>
@@ -851,8 +880,11 @@
       <c r="H8" s="21" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="9" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="I8" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D9" s="22">
         <v>5</v>
       </c>
@@ -868,8 +900,11 @@
       <c r="H9" s="23" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="I9" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D10" s="24">
         <v>6</v>
       </c>
@@ -879,10 +914,14 @@
       <c r="F10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="25"/>
-    </row>
-    <row r="11" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D11" s="26">
         <v>7</v>
       </c>
@@ -892,10 +931,14 @@
       <c r="F11" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="27"/>
-    </row>
-    <row r="12" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G11" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D12" s="28">
         <v>8</v>
       </c>
@@ -905,10 +948,14 @@
       <c r="F12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="9"/>
-      <c r="H12" s="29"/>
-    </row>
-    <row r="13" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G12" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H12" s="29" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D13" s="35">
         <v>9</v>
       </c>
@@ -925,7 +972,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D14" s="35">
         <v>10</v>
       </c>
@@ -942,7 +989,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D15" s="22">
         <v>11</v>
       </c>
@@ -955,7 +1002,7 @@
       <c r="G15" s="6"/>
       <c r="H15" s="23"/>
     </row>
-    <row r="16" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D16" s="24">
         <v>12</v>
       </c>

</xml_diff>